<commit_message>
Contrato con desgloses, nota y estado; README apunta a la Entrega 1; diccionario: población por comuna = Censo 2022
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
+++ b/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
@@ -1077,7 +1077,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>https://cdn.buenosaires.gob.ar/datosabiertos/datasets/barrios/caba_pob_barrios_2010.csv ; https://cdn.buenosaires.gob.ar/datosabiertos/datasets/comunas/gcba_pob_comunas_17.csv</t>
+          <t>https://cdn.buenosaires.gob.ar/datosabiertos/datasets/barrios/caba_pob_barrios_2010.csv</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -1102,12 +1102,12 @@
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>Barrios y comunas</t>
+          <t>Ciudad, 48 barrios</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>Censo 2010 (barrios); proyección 2017 (comunas)</t>
+          <t>Censo 2010</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>habitantes</t>
+          <t>habitantes (Censo 2010)</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
@@ -10114,7 +10114,7 @@
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -10129,12 +10129,12 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>COMUNA, POBLACION</t>
+          <t>Anexo 1, cuadro C.1 (PDF)</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Habitantes de cada comuna (proyección 2017 del portal) (desglose [categoría, valor])</t>
+          <t>Habitantes de cada comuna en el Censo 2022 (desglose [categoría, valor])</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>habitantes</t>
+          <t>habitantes (Censo 2022 definitivo)</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="L49" s="10" t="inlineStr">
         <is>
-          <t>Se copia</t>
+          <t>Transcrito del PDF a ingesta/datos/censo2022_comunas.csv; la suma = total oficial</t>
         </is>
       </c>
       <c r="M49" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Entrega 1: documento «Por qué estos datos» lleno desde el lago; bitácora IA cita F35 y F33
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
+++ b/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
@@ -18836,7 +18836,11 @@
           <t>Incorrecto</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Que exista un conjunto con el nombre correcto no quiere decir que tenga el año que se necesita.</t>
@@ -18912,7 +18916,11 @@
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>F33</t>
+        </is>
+      </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
           <t>La causa de un hueco también se verifica: el motivo anotado era otro.</t>

</xml_diff>

<commit_message>
Entrega 1: integrantes (Jacobo Montes Castaño y Carlos Restrepo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
+++ b/entrega/Diccionario_de_datos_Buenos_Aires.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21620" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1. Fuentes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2. Diccionario" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3. Bitácora IA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Fuentes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Diccionario" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Bitácora IA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -581,7 +581,7 @@
     <row r="6">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Integrantes:</t>
+          <t>Integrantes: Jacobo Montes Castaño y Carlos Restrepo</t>
         </is>
       </c>
     </row>
@@ -21136,7 +21136,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>

</xml_diff>